<commit_message>
Reclassify Data/UI/Visual Consistency as Current Feature Enhancement
https://claude.ai/code/session_01Yc1FCZVYdn8PdJ2AcRFkWB
</commit_message>
<xml_diff>
--- a/app_issues_backlog.xlsx
+++ b/app_issues_backlog.xlsx
@@ -2222,7 +2222,6 @@
           <t>APP ISSUES BACKLOG — STOMASENSE</t>
         </is>
       </c>
-      <c r="P1" s="58" t="n"/>
     </row>
     <row r="2" ht="20.1" customHeight="1" s="61">
       <c r="A2" s="53" t="inlineStr">
@@ -2230,7 +2229,6 @@
           <t>Total Issues: 103  |  Resolved: 103  |  Open: 0  |  Pre-March 2026 items marked as Resolved</t>
         </is>
       </c>
-      <c r="P2" s="59" t="n"/>
     </row>
     <row r="3" ht="27.95" customHeight="1" s="61">
       <c r="A3" s="30" t="inlineStr">
@@ -2578,7 +2576,7 @@
       </c>
       <c r="F7" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G7" s="50" t="n">
@@ -3040,7 +3038,7 @@
       </c>
       <c r="F13" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G13" s="50" t="n">
@@ -3502,7 +3500,7 @@
       </c>
       <c r="F19" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G19" s="50" t="n">
@@ -4811,7 +4809,7 @@
       </c>
       <c r="F36" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G36" s="49" t="n">
@@ -4888,7 +4886,7 @@
       </c>
       <c r="F37" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G37" s="50" t="n">
@@ -5735,7 +5733,7 @@
       </c>
       <c r="F48" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G48" s="49" t="n">
@@ -5810,7 +5808,7 @@
       </c>
       <c r="F49" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G49" s="50" t="n">
@@ -5886,7 +5884,7 @@
       </c>
       <c r="F50" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G50" s="49" t="n">
@@ -6261,7 +6259,7 @@
       </c>
       <c r="F55" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G55" s="50" t="n">
@@ -6336,7 +6334,7 @@
       </c>
       <c r="F56" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G56" s="49" t="n">
@@ -6486,7 +6484,7 @@
       </c>
       <c r="F58" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G58" s="49" t="n">
@@ -6561,7 +6559,7 @@
       </c>
       <c r="F59" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G59" s="50" t="n">
@@ -6636,7 +6634,7 @@
       </c>
       <c r="F60" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G60" s="49" t="n">
@@ -7012,7 +7010,7 @@
       </c>
       <c r="F65" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G65" s="50" t="n">
@@ -7087,7 +7085,7 @@
       </c>
       <c r="F66" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G66" s="49" t="n">
@@ -7164,7 +7162,7 @@
       </c>
       <c r="F67" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G67" s="50" t="n">
@@ -7316,7 +7314,7 @@
       </c>
       <c r="F69" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G69" s="50" t="n">
@@ -7698,7 +7696,7 @@
       </c>
       <c r="F74" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G74" s="49" t="n">
@@ -7775,7 +7773,7 @@
       </c>
       <c r="F75" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G75" s="50" t="n">
@@ -8375,7 +8373,7 @@
       </c>
       <c r="F83" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G83" s="50" t="n">
@@ -9275,7 +9273,7 @@
       </c>
       <c r="F95" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G95" s="50" t="n">
@@ -9350,7 +9348,7 @@
       </c>
       <c r="F96" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G96" s="49" t="n">
@@ -9811,7 +9809,7 @@
       </c>
       <c r="F102" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G102" s="49" t="n">
@@ -9886,7 +9884,7 @@
       </c>
       <c r="F103" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G103" s="50" t="n">
@@ -11280,7 +11278,7 @@
       </c>
       <c r="F121" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G121" s="50" t="n">
@@ -11434,7 +11432,7 @@
       </c>
       <c r="F123" s="65" t="inlineStr">
         <is>
-          <t>Issues and Bugs</t>
+          <t>Current Feature Enhancement</t>
         </is>
       </c>
       <c r="G123" s="50" t="n">

</xml_diff>